<commit_message>
updated Template for SBL mandate report
</commit_message>
<xml_diff>
--- a/reporting/report_template/SBL_CLO_100_Template.xlsx
+++ b/reporting/report_template/SBL_CLO_100_Template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\XiaHanlu\workspace\legacyReporting\reporting\report_template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC783897-2FA0-4B08-B7B2-9ED0BAC2019C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{358E9E10-530C-4975-834A-0289213895E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6135,6 +6135,79 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="168" formatCode="0.0"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+      </border>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
       <numFmt numFmtId="168" formatCode="0.0"/>
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -6156,7 +6229,59 @@
         <scheme val="none"/>
       </font>
       <numFmt numFmtId="168" formatCode="0.0"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+      </border>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="168" formatCode="0.0"/>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -6229,17 +6354,11 @@
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
         <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
         <name val="Arial"/>
         <family val="2"/>
         <scheme val="none"/>
@@ -6260,60 +6379,6 @@
       </font>
       <numFmt numFmtId="14" formatCode="0.00%"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="168" formatCode="0.0"/>
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -6341,26 +6406,6 @@
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="168" formatCode="0.0"/>
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
         <strike val="0"/>
         <condense val="0"/>
         <extend val="0"/>
@@ -6382,25 +6427,6 @@
         </patternFill>
       </fill>
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -11725,22 +11751,22 @@
 </file>
 
 <file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{12D42117-5193-441A-8C14-66A40D5E97B1}" name="Table20" displayName="Table20" ref="H26:L37" totalsRowCount="1" headerRowDxfId="56" dataDxfId="55" totalsRowDxfId="54">
-  <autoFilter ref="H26:L36" xr:uid="{12D42117-5193-441A-8C14-66A40D5E97B1}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{12D42117-5193-441A-8C14-66A40D5E97B1}" name="Table20" displayName="Table20" ref="H26:L38" totalsRowCount="1" headerRowDxfId="56" dataDxfId="55" totalsRowDxfId="54">
+  <autoFilter ref="H26:L37" xr:uid="{12D42117-5193-441A-8C14-66A40D5E97B1}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{2727D7D5-D5F7-4EE8-96FD-6A1A9AB27A40}" name="Vintage" totalsRowLabel="Total" dataDxfId="53" totalsRowDxfId="52"/>
-    <tableColumn id="2" xr3:uid="{C11EED73-564D-45E3-BA47-0F6B94FCFA00}" name="Current Face (M)" totalsRowFunction="sum" dataDxfId="51" totalsRowDxfId="50" dataCellStyle="Percent" totalsRowCellStyle="Percent">
+    <tableColumn id="1" xr3:uid="{2727D7D5-D5F7-4EE8-96FD-6A1A9AB27A40}" name="Vintage" totalsRowLabel="Total" dataDxfId="53" totalsRowDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{C11EED73-564D-45E3-BA47-0F6B94FCFA00}" name="Current Face (M)" totalsRowFunction="sum" dataDxfId="52" totalsRowDxfId="3" dataCellStyle="Percent">
       <calculatedColumnFormula>Table20[[#This Row],[Portfolio % CF]]*$C$10/1000000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{9A8F8B71-DCBA-41AB-9C93-D8D1AA49B14C}" name="Market Value (M)" totalsRowFunction="sum" dataDxfId="49" totalsRowDxfId="48" dataCellStyle="Percent" totalsRowCellStyle="Percent">
+    <tableColumn id="3" xr3:uid="{9A8F8B71-DCBA-41AB-9C93-D8D1AA49B14C}" name="Market Value (M)" totalsRowFunction="sum" dataDxfId="51" totalsRowDxfId="2" dataCellStyle="Percent">
       <calculatedColumnFormula>Table20[[#This Row],[Portfolio % MV]]*$C$11/1000000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{18762466-9940-404E-B47A-2FC91F086CD5}" name="Portfolio % CF" totalsRowFunction="sum" dataDxfId="47" totalsRowDxfId="46" dataCellStyle="Percent">
+    <tableColumn id="4" xr3:uid="{18762466-9940-404E-B47A-2FC91F086CD5}" name="Portfolio % CF" totalsRowFunction="sum" dataDxfId="50" totalsRowDxfId="1" dataCellStyle="Percent">
       <calculatedColumnFormula>IFERROR(IF($C$4="All Portfolios",
    SUMIFS(Positions!$C$2:$C$644,tbl_rawhold[Vintage],Table20[[#This Row],[Vintage]])/$C$10,
    SUMIFS(Positions!$C$2:$C$644,tbl_rawhold[Vintage],Table20[[#This Row],[Vintage]],Positions!$M$2:$M$644,$C$4)/$C$10),0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{82838F31-AA15-4535-929C-0E3A529E0EBF}" name="Portfolio % MV" totalsRowFunction="sum" dataDxfId="45" totalsRowDxfId="44" dataCellStyle="Percent">
+    <tableColumn id="5" xr3:uid="{82838F31-AA15-4535-929C-0E3A529E0EBF}" name="Portfolio % MV" totalsRowFunction="sum" dataDxfId="49" totalsRowDxfId="0" dataCellStyle="Percent">
       <calculatedColumnFormula>IFERROR(IF($C$4="All Portfolios",
    SUMIFS(Positions!$D$2:$D$644,tbl_rawhold[Vintage],Table20[[#This Row],[Vintage]])/$C$11,
    SUMIFS(Positions!$D$2:$D$644,tbl_rawhold[Vintage],Table20[[#This Row],[Vintage]],Positions!$M$2:$M$644,$C$4)/$C$11),0)</calculatedColumnFormula>
@@ -11751,22 +11777,22 @@
 </file>
 
 <file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="21" xr:uid="{27E8DB96-6F30-4B07-B6B9-321E95208A1F}" name="Table21" displayName="Table21" ref="N26:R33" totalsRowCount="1" headerRowDxfId="43" dataDxfId="42" totalsRowDxfId="41" dataCellStyle="Percent">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="21" xr:uid="{27E8DB96-6F30-4B07-B6B9-321E95208A1F}" name="Table21" displayName="Table21" ref="N26:R33" totalsRowCount="1" headerRowDxfId="48" dataDxfId="47" totalsRowDxfId="46" dataCellStyle="Percent">
   <autoFilter ref="N26:R32" xr:uid="{27E8DB96-6F30-4B07-B6B9-321E95208A1F}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{C0E68083-58A0-4469-8380-6EFE6E688032}" name="Collateral Type" totalsRowLabel="Total" dataDxfId="40" totalsRowDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{B110CD2D-60E4-4123-9297-9C7E7830F08A}" name="Current Face (M)" totalsRowFunction="sum" dataDxfId="39" totalsRowDxfId="3" dataCellStyle="Percent">
+    <tableColumn id="1" xr3:uid="{C0E68083-58A0-4469-8380-6EFE6E688032}" name="Collateral Type" totalsRowLabel="Total" dataDxfId="45" totalsRowDxfId="44"/>
+    <tableColumn id="2" xr3:uid="{B110CD2D-60E4-4123-9297-9C7E7830F08A}" name="Current Face (M)" totalsRowFunction="sum" dataDxfId="43" totalsRowDxfId="42" dataCellStyle="Percent">
       <calculatedColumnFormula>Table21[[#This Row],[Portfolio % CF]]*$C$10/1000000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{37038776-57D1-43F8-BD18-FDFAF46F9CD9}" name="Market Value (M)" totalsRowFunction="sum" dataDxfId="38" totalsRowDxfId="2" dataCellStyle="Percent">
+    <tableColumn id="3" xr3:uid="{37038776-57D1-43F8-BD18-FDFAF46F9CD9}" name="Market Value (M)" totalsRowFunction="sum" dataDxfId="41" totalsRowDxfId="40" dataCellStyle="Percent">
       <calculatedColumnFormula>Table21[[#This Row],[Portfolio % MV]]*$C$11/1000000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{A8F097ED-132B-4894-8D01-8D0EB3526B1D}" name="Portfolio % CF" totalsRowFunction="sum" dataDxfId="37" totalsRowDxfId="1" dataCellStyle="Percent">
+    <tableColumn id="4" xr3:uid="{A8F097ED-132B-4894-8D01-8D0EB3526B1D}" name="Portfolio % CF" totalsRowFunction="sum" dataDxfId="39" totalsRowDxfId="38" dataCellStyle="Percent">
       <calculatedColumnFormula>IFERROR(IF($C$4="All Portfolios",
    SUMIFS(Positions!$C$2:$C$644,tbl_rawhold[Collateral Type],Table21[[#This Row],[Collateral Type]])/$C$10,
    SUMIFS(Positions!$C$2:$C$644,tbl_rawhold[Collateral Type],Table21[[#This Row],[Collateral Type]],Positions!$M$2:$M$644,$C$4)/$C$10),0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{26DD84D2-9931-4777-99E2-3808183B7A4E}" name="Portfolio % MV" totalsRowFunction="sum" dataDxfId="36" totalsRowDxfId="0" dataCellStyle="Percent">
+    <tableColumn id="5" xr3:uid="{26DD84D2-9931-4777-99E2-3808183B7A4E}" name="Portfolio % MV" totalsRowFunction="sum" dataDxfId="37" totalsRowDxfId="36" dataCellStyle="Percent">
       <calculatedColumnFormula>IFERROR(IF($C$4="All Portfolios",
    SUMIFS(Positions!$D$2:$D$644,tbl_rawhold[Collateral Type],Table21[[#This Row],[Collateral Type]])/$C$11,
    SUMIFS(Positions!$D$2:$D$644,tbl_rawhold[Collateral Type],Table21[[#This Row],[Collateral Type]],Positions!$M$2:$M$644,$C$4)/$C$11),0)</calculatedColumnFormula>
@@ -12952,7 +12978,7 @@
     </row>
     <row r="4" spans="2:15" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B4" s="2">
-        <v>45869</v>
+        <v>46142</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>4</v>
@@ -14169,8 +14195,8 @@
       <c r="R35" s="20"/>
     </row>
     <row r="36" spans="2:18" x14ac:dyDescent="0.2">
-      <c r="H36" s="17" t="s">
-        <v>1650</v>
+      <c r="H36" s="17">
+        <v>2026</v>
       </c>
       <c r="I36" s="51">
         <f>Table20[[#This Row],[Portfolio % CF]]*$C$10/1000000</f>
@@ -14195,29 +14221,49 @@
     </row>
     <row r="37" spans="2:18" x14ac:dyDescent="0.2">
       <c r="H37" s="17" t="s">
+        <v>1650</v>
+      </c>
+      <c r="I37" s="46">
+        <f>Table20[[#This Row],[Portfolio % CF]]*$C$10/1000000</f>
+        <v>0</v>
+      </c>
+      <c r="J37" s="46">
+        <f>Table20[[#This Row],[Portfolio % MV]]*$C$11/1000000</f>
+        <v>0</v>
+      </c>
+      <c r="K37" s="20">
+        <f>IFERROR(IF($C$4="All Portfolios",
+   SUMIFS(Positions!$C$2:$C$644,tbl_rawhold[Vintage],Table20[[#This Row],[Vintage]])/$C$10,
+   SUMIFS(Positions!$C$2:$C$644,tbl_rawhold[Vintage],Table20[[#This Row],[Vintage]],Positions!$M$2:$M$644,$C$4)/$C$10),0)</f>
+        <v>0</v>
+      </c>
+      <c r="L37" s="20">
+        <f>IFERROR(IF($C$4="All Portfolios",
+   SUMIFS(Positions!$D$2:$D$644,tbl_rawhold[Vintage],Table20[[#This Row],[Vintage]])/$C$11,
+   SUMIFS(Positions!$D$2:$D$644,tbl_rawhold[Vintage],Table20[[#This Row],[Vintage]],Positions!$M$2:$M$644,$C$4)/$C$11),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="2:18" x14ac:dyDescent="0.2">
+      <c r="H38" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="I37" s="50">
+      <c r="I38" s="50">
         <f>SUBTOTAL(109,Table20[Current Face (M)])</f>
         <v>3070.3171847427634</v>
       </c>
-      <c r="J37" s="50">
+      <c r="J38" s="50">
         <f>SUBTOTAL(109,Table20[Market Value (M)])</f>
         <v>3046.1577266000004</v>
       </c>
-      <c r="K37" s="16">
+      <c r="K38" s="16">
         <f>SUBTOTAL(109,Table20[Portfolio % CF])</f>
         <v>1.713302703016617</v>
       </c>
-      <c r="L37" s="16">
+      <c r="L38" s="16">
         <f>SUBTOTAL(109,Table20[Portfolio % MV])</f>
         <v>1.7233927439292949</v>
       </c>
-    </row>
-    <row r="38" spans="2:18" x14ac:dyDescent="0.2">
-      <c r="I38" s="17"/>
-      <c r="J38" s="16"/>
-      <c r="K38" s="16"/>
     </row>
     <row r="39" spans="2:18" x14ac:dyDescent="0.2">
       <c r="I39" s="17"/>

</xml_diff>